<commit_message>
Update template xlsx file
</commit_message>
<xml_diff>
--- a/www/samples/FD-048BL - sample.xlsx
+++ b/www/samples/FD-048BL - sample.xlsx
@@ -5680,7 +5680,7 @@
     <numFmt numFmtId="165" formatCode="@"/>
     <numFmt numFmtId="166" formatCode="#,##0.00"/>
   </numFmts>
-  <fonts count="10">
+  <fonts count="9">
     <font>
       <sz val="10"/>
       <color rgb="FF000000"/>
@@ -5704,16 +5704,9 @@
       <family val="0"/>
     </font>
     <font>
-      <sz val="10"/>
-      <color rgb="FFFFFFFF"/>
-      <name val="Arial"/>
-      <family val="0"/>
-      <charset val="1"/>
-    </font>
-    <font>
       <b val="true"/>
       <sz val="10"/>
-      <color rgb="FFFFFFFF"/>
+      <color rgb="FF000000"/>
       <name val="Arial"/>
       <family val="0"/>
       <charset val="1"/>
@@ -5721,7 +5714,7 @@
     <font>
       <b val="true"/>
       <sz val="8"/>
-      <color rgb="FFFFFFFF"/>
+      <color rgb="FF000000"/>
       <name val="Arial"/>
       <family val="0"/>
       <charset val="1"/>
@@ -5730,7 +5723,7 @@
       <b val="true"/>
       <i val="true"/>
       <sz val="10"/>
-      <color rgb="FFFFFFFF"/>
+      <color rgb="FF000000"/>
       <name val="Arial"/>
       <family val="0"/>
       <charset val="1"/>
@@ -5738,14 +5731,14 @@
     <font>
       <b val="true"/>
       <sz val="9"/>
-      <color rgb="FFFFFFFF"/>
+      <color rgb="FF000000"/>
       <name val="Arial"/>
       <family val="0"/>
       <charset val="1"/>
     </font>
     <font>
       <sz val="9"/>
-      <color rgb="FFFFFFFF"/>
+      <color rgb="FF000000"/>
       <name val="Arial"/>
       <family val="0"/>
       <charset val="1"/>
@@ -5811,71 +5804,71 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="right" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="165" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="165" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="4" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="4" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="166" fontId="4" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="166" fontId="0" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>

</xml_diff>